<commit_message>
adapt MC for mode_Inertia
</commit_message>
<xml_diff>
--- a/RocketPy_26_MC/DEFAULT.xlsx
+++ b/RocketPy_26_MC/DEFAULT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/085522fb5f488138/Documents/GitHub/2026_C_FD_SIM_Rocketpy/RocketPy_26_MC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="11_027D8733D211528E904E752E17EFE3F86DEECCEB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28E85AB0-3DB1-4FAE-9535-6F698A54296F}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="11_027D8733D211528E904E752E17EFE3F86DEECCEB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3050C198-AE5E-4AB0-B185-370F98F9E527}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4356" yWindow="5100" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="144">
   <si>
     <t>Name</t>
   </si>
@@ -34,9 +34,6 @@
     <t>ROCKET</t>
   </si>
   <si>
-    <t>mode</t>
-  </si>
-  <si>
     <t>l_center_of_mass</t>
   </si>
   <si>
@@ -452,6 +449,12 @@
   </si>
   <si>
     <t>lox_pressure</t>
+  </si>
+  <si>
+    <t>mode_CoM</t>
+  </si>
+  <si>
+    <t>mode_Inertia</t>
   </si>
 </sst>
 </file>
@@ -511,6 +514,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -798,7 +805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B70"/>
+  <dimension ref="A1:B71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -820,7 +827,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>142</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -828,495 +835,503 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>143</v>
       </c>
       <c r="B4">
-        <v>266</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B5">
-        <v>84500</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6">
-        <v>0.1215</v>
+        <v>84500</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>0.1215</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="B7">
-        <v>0.38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>0.1215</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B10">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1215</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B11">
-        <v>0.41754999999999998</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>0.41754999999999998</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>4.9459999999999997E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B13">
-        <v>4.9459999999999997E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15">
-        <v>0.75600000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>0.75600000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>26.475999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B16">
-        <v>26.475999999999999</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18">
-        <v>1.393</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B19">
-        <v>0.38800000000000001</v>
+        <v>1.393</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>0.38800000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>8.3870000000000005</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B20">
-        <v>8.3870000000000005</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22">
-        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B23">
-        <v>2.41</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B24">
-        <v>1.6557999999999999</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25">
+        <v>1.6557999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B25">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>27</v>
-      </c>
-      <c r="B27">
-        <v>2.2253099999999999</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B28">
-        <v>0.9</v>
+        <v>2.2253099999999999</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30">
+        <v>11.048999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B29">
-        <v>11.048999999999999</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31">
-        <v>2.9980000000000002</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B32">
-        <v>0.38800000000000001</v>
+        <v>2.9980000000000002</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33">
+        <v>0.38800000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34">
+        <v>8.3870000000000005</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B33">
-        <v>8.3870000000000005</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>35</v>
-      </c>
-      <c r="B35">
-        <v>3.6473100000000001</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B36">
-        <v>0.9</v>
+        <v>3.6473100000000001</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38">
+        <v>11.03</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B37">
-        <v>11.03</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>39</v>
-      </c>
-      <c r="B39">
-        <v>0.35</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41">
+        <v>9.2319999999999993</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="B40">
-        <v>9.2319999999999993</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>42</v>
-      </c>
-      <c r="B42">
-        <v>0.71499999999999997</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B43">
-        <v>11.044</v>
+        <v>0.71499999999999997</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B44">
-        <v>4</v>
+        <v>11.044</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B45">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>45</v>
+      </c>
+      <c r="B47">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B46">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>48</v>
-      </c>
-      <c r="B48">
-        <v>1.0029999999999999</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>47</v>
+      </c>
+      <c r="B49">
+        <v>1.0029999999999999</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50">
+        <v>5.8380000000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="B49">
-        <v>5.8380000000000001</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>51</v>
-      </c>
-      <c r="B51">
-        <v>0.115</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>52</v>
-      </c>
-      <c r="B52" t="s">
-        <v>53</v>
+        <v>50</v>
+      </c>
+      <c r="B52">
+        <v>0.115</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>54</v>
-      </c>
-      <c r="B53">
-        <v>1.6E-2</v>
+        <v>51</v>
+      </c>
+      <c r="B53" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>1.6E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="B54">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>57</v>
-      </c>
-      <c r="B56">
-        <v>8.5800000000000001E-2</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>58</v>
-      </c>
-      <c r="B57" t="s">
-        <v>53</v>
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>8.5800000000000001E-2</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>8.9999999999999993E-3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="B58">
-        <v>8.9999999999999993E-3</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>61</v>
-      </c>
-      <c r="B60">
-        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B61">
-        <v>0.3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B62">
-        <v>0.67100000000000004</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B63">
-        <v>0.161</v>
+        <v>0.67100000000000004</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B64">
-        <v>1.1315</v>
+        <v>0.161</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B65">
-        <v>0</v>
+        <v>1.1315</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B66">
-        <v>0.53900000000000003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>66</v>
+      </c>
+      <c r="B67">
+        <v>0.53900000000000003</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <v>2.4187859999999999</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="B67">
-        <v>2.4187859999999999</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>70</v>
-      </c>
-      <c r="B69">
-        <v>0.46279999999999999</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B70">
+        <v>0.46279999999999999</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>70</v>
+      </c>
+      <c r="B71">
         <v>0.46278999999999998</v>
       </c>
     </row>
@@ -1344,12 +1359,12 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B3">
         <v>1.5</v>
@@ -1357,7 +1372,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B4">
         <v>190</v>
@@ -1365,7 +1380,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B5">
         <v>7000</v>
@@ -1373,7 +1388,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B6">
         <v>36000</v>
@@ -1381,20 +1396,20 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
         <v>78</v>
-      </c>
-      <c r="B8" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -1402,12 +1417,12 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B11">
         <v>1E-3</v>
@@ -1415,7 +1430,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B12">
         <v>4.3620000000000001</v>
@@ -1423,7 +1438,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B13">
         <v>4.3620000000000001</v>
@@ -1431,7 +1446,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B14">
         <v>2.6231688709999998</v>
@@ -1439,7 +1454,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B15">
         <v>2.6231688709999998</v>
@@ -1447,7 +1462,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B16">
         <v>3.634769409</v>
@@ -1455,7 +1470,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1463,7 +1478,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B18">
         <v>1.672500989</v>
@@ -1471,7 +1486,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B19">
         <v>1.672500989</v>
@@ -1479,7 +1494,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B20">
         <v>2.2932178200000002</v>
@@ -1487,7 +1502,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B21">
         <v>7.4999999999999997E-2</v>
@@ -1495,12 +1510,12 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B23">
         <v>293.14999999999998</v>
@@ -1508,7 +1523,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B24" s="2">
         <v>6000000</v>
@@ -1516,7 +1531,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B25" s="2">
         <v>0.9</v>
@@ -1524,7 +1539,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B26">
         <v>0.40500000000000003</v>
@@ -1532,7 +1547,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B27">
         <v>90.15</v>
@@ -1540,7 +1555,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B28" s="2">
         <v>6000000</v>
@@ -1548,7 +1563,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B29">
         <v>0.57699999999999996</v>
@@ -1556,7 +1571,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B30">
         <v>2.605</v>
@@ -1564,12 +1579,12 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B32">
         <v>300</v>
@@ -1577,7 +1592,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B33">
         <v>0.2</v>
@@ -1585,7 +1600,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B34">
         <v>-0.05</v>
@@ -1593,7 +1608,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B35">
         <v>0.4</v>
@@ -1601,7 +1616,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B36">
         <v>0.2</v>
@@ -1609,7 +1624,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B37">
         <v>2.5000000000000001E-2</v>
@@ -1617,12 +1632,12 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -1630,7 +1645,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B40">
         <v>3300</v>
@@ -1660,28 +1675,28 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" t="s">
         <v>108</v>
-      </c>
-      <c r="B3" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B5">
         <v>1000</v>
@@ -1689,81 +1704,81 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" t="s">
         <v>114</v>
-      </c>
-      <c r="B8" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B16">
         <v>2026</v>
@@ -1771,7 +1786,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B17">
         <v>6</v>
@@ -1779,7 +1794,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B18">
         <v>2</v>
@@ -1787,7 +1802,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B19">
         <v>12</v>
@@ -1795,7 +1810,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1803,7 +1818,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B21">
         <v>39.390149999999998</v>
@@ -1811,7 +1826,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B22">
         <v>-8.2891449999999995</v>
@@ -1819,7 +1834,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B23">
         <v>130</v>
@@ -1827,12 +1842,12 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B25">
         <v>6</v>
@@ -1840,7 +1855,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B26">
         <v>6</v>
@@ -1848,7 +1863,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B27">
         <v>11.65</v>
@@ -1856,7 +1871,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B28">
         <v>0.5</v>
@@ -1864,7 +1879,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B29">
         <v>84</v>
@@ -1872,7 +1887,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B30">
         <v>144</v>

</xml_diff>

<commit_message>
adjust MC for multiple columns with mode_com
</commit_message>
<xml_diff>
--- a/RocketPy_26_MC/DEFAULT.xlsx
+++ b/RocketPy_26_MC/DEFAULT.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/085522fb5f488138/Documents/GitHub/2026_C_FD_SIM_Rocketpy/RocketPy_26_MC/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_027D8733D211528E904E752E17EFE3F86DEECCEB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3050C198-AE5E-4AB0-B185-370F98F9E527}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_C40B6BE15FF3DC814638DB4B9633989B1F4717A0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDFB8CF5-5153-44D7-A0C5-598E6396F435}"/>
   <bookViews>
-    <workbookView xWindow="4356" yWindow="5100" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" r:id="rId1"/>
@@ -18,12 +13,12 @@
     <sheet name="Parameters " sheetId="3" r:id="rId3"/>
     <sheet name="Simulation" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="145">
   <si>
     <t>Name</t>
   </si>
@@ -31,9 +26,18 @@
     <t>Value</t>
   </si>
   <si>
+    <t>Value (mass) for mode_CoM == 1</t>
+  </si>
+  <si>
     <t>ROCKET</t>
   </si>
   <si>
+    <t>mode_CoM</t>
+  </si>
+  <si>
+    <t>mode_Inertia</t>
+  </si>
+  <si>
     <t>l_center_of_mass</t>
   </si>
   <si>
@@ -304,9 +308,24 @@
     <t>MASS</t>
   </si>
   <si>
+    <t>eth_temperature</t>
+  </si>
+  <si>
+    <t>eth_pressure</t>
+  </si>
+  <si>
+    <t>eth_massic_frac</t>
+  </si>
+  <si>
     <t>m_eth_unused</t>
   </si>
   <si>
+    <t>lox_temperature</t>
+  </si>
+  <si>
+    <t>lox_pressure</t>
+  </si>
+  <si>
     <t>m_lox_unused</t>
   </si>
   <si>
@@ -434,27 +453,6 @@
   </si>
   <si>
     <t>heading_rail</t>
-  </si>
-  <si>
-    <t>eth_temperature</t>
-  </si>
-  <si>
-    <t>eth_pressure</t>
-  </si>
-  <si>
-    <t>eth_massic_frac</t>
-  </si>
-  <si>
-    <t>lox_temperature</t>
-  </si>
-  <si>
-    <t>lox_pressure</t>
-  </si>
-  <si>
-    <t>mode_CoM</t>
-  </si>
-  <si>
-    <t>mode_Inertia</t>
   </si>
 </sst>
 </file>
@@ -504,7 +502,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -514,10 +512,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -805,531 +799,568 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B71"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C71"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>142</v>
+        <v>4</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>143</v>
+        <v>5</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B5">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>2.66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B6">
-        <v>84500</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+        <v>84.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0.1215</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0.38</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B10">
         <v>0.1215</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B11">
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B12">
         <v>0.41754999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>7.3529999999999998</v>
+      </c>
+      <c r="C13">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>4.9459999999999997E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B16">
         <v>0.75600000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B17">
-        <v>26.475999999999999</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+        <v>12.797000000000001</v>
+      </c>
+      <c r="C17">
+        <v>2.6463999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B19">
         <v>1.393</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B20">
         <v>0.38800000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B21">
         <v>8.3870000000000005</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B23">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B24">
-        <v>2.41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+        <v>2.38</v>
+      </c>
+      <c r="C24">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B25">
         <v>1.6557999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B26">
         <v>0.03</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B28">
         <v>2.2253099999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B29">
         <v>0.9</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B30">
-        <v>11.048999999999999</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+        <v>17.527000000000001</v>
+      </c>
+      <c r="C30">
+        <v>1.7527999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B32">
         <v>2.9980000000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B33">
         <v>0.38800000000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B34">
         <v>8.3870000000000005</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B36">
         <v>3.6473100000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B37">
         <v>0.9</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B38">
-        <v>11.03</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+        <v>14.21</v>
+      </c>
+      <c r="C38">
+        <v>1.2154</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B40">
         <v>0.35</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B41">
-        <v>9.2319999999999993</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+        <v>9.8350000000000009</v>
+      </c>
+      <c r="C41">
+        <v>0.54279999999999995</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B43">
         <v>0.71499999999999997</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B44">
-        <v>11.044</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+        <v>10.311</v>
+      </c>
+      <c r="C44">
+        <v>0.2054</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B45">
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B46">
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B47">
         <v>400</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B49">
         <v>1.0029999999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B50">
-        <v>5.8380000000000001</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+        <v>5.6120000000000001</v>
+      </c>
+      <c r="C50">
+        <v>3.6829999999999998</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B52">
         <v>0.115</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B54">
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B55">
         <v>0.05</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B57">
         <v>8.5800000000000001E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B59">
         <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B61">
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B62">
         <v>0.3</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B63">
         <v>0.67100000000000004</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B64">
         <v>0.161</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B65">
         <v>1.1315</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B66">
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B67">
         <v>0.53900000000000003</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B68">
-        <v>2.4187859999999999</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+        <v>2.4</v>
+      </c>
+      <c r="C68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B70">
         <v>0.46279999999999999</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B71">
         <v>0.46278999999999998</v>
@@ -1343,13 +1374,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1357,295 +1388,295 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B3">
         <v>1.5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B4">
         <v>190</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B5">
         <v>7000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B6">
         <v>36000</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B9">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B11">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B12">
         <v>4.3620000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B13">
         <v>4.3620000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B14">
         <v>2.6231688709999998</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B15">
         <v>2.6231688709999998</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B16">
         <v>3.634769409</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B18">
         <v>1.672500989</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B19">
         <v>1.672500989</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B20">
         <v>2.2932178200000002</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B21">
         <v>7.4999999999999997E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>137</v>
+        <v>96</v>
       </c>
       <c r="B23">
         <v>293.14999999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>138</v>
+        <v>97</v>
       </c>
       <c r="B24" s="2">
         <v>6000000</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>139</v>
+        <v>98</v>
       </c>
       <c r="B25" s="2">
         <v>0.9</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B26">
         <v>0.40500000000000003</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="B27">
         <v>90.15</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>141</v>
+        <v>101</v>
       </c>
       <c r="B28" s="2">
         <v>6000000</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="B29">
         <v>0.57699999999999996</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="B30">
         <v>2.605</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B32">
         <v>300</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="B33">
         <v>0.2</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="B34">
         <v>-0.05</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="B35">
         <v>0.4</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B36">
         <v>0.2</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B37">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B39">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B40">
         <v>3300</v>
@@ -1659,13 +1690,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1673,221 +1704,221 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="B5">
         <v>1000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="B12" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B16">
         <v>2026</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B17">
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B18">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B19">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="B20">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B21">
         <v>39.390149999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B22">
         <v>-8.2891449999999995</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B23">
         <v>130</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="B25">
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B26">
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B27">
         <v>11.65</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="B28">
         <v>0.5</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B29">
         <v>84</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="B30">
         <v>144</v>
@@ -1901,9 +1932,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>

</xml_diff>